<commit_message>
Update validatieregel-tabel 1.5 met nieuwe toelichtingen
</commit_message>
<xml_diff>
--- a/validation_rules/overzichten_ValidationRules/overzicht_ValidationRules_1.4.xlsx
+++ b/validation_rules/overzichten_ValidationRules/overzicht_ValidationRules_1.4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="ValidationRules_1.4" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ValidationRules_1.4'!$A$1:$H$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ValidationRules_1.4'!$A$1:$H$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>left=maximalehoogteopening, right=kunstwerkopening_hoogte_m</t>
+          <t>left=hoogteopening, right=kunstwerkopening_hoogte_m</t>
         </is>
       </c>
     </row>
@@ -2805,12 +2805,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>general_001_kunstwerkopening_laagstedoorstroomhoogte</t>
+          <t>general_001_doorstroomopening_laagstedoorstroomhoogte</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Berekening van 'kunstwerkopening_laagstedoorstroomhoogte'</t>
+          <t>Berekening van 'doorstroomopening_laagstedoorstroomhoogte'</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>statistic=min, related_object=kunstwerkopening, related_parameter=laagstedoorstroomhoogte</t>
+          <t>statistic=min, related_object=doorstroomopening, related_parameter=laagstedoorstroomhoogte</t>
         </is>
       </c>
     </row>
@@ -2842,22 +2842,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>general_002_kunstwerkopening_laagstedoorstroombreedte</t>
+          <t>validate_000_hoogtebovenzijde_plausibel</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Berekening van 'kunstwerkopening_laagstedoorstroombreedte'</t>
+          <t>hoogtebovenzijde plausibel (-8m - 325m)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2867,12 +2867,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
+          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>statistic=sum, related_object=kunstwerkopening, related_parameter=laagstedoorstroombreedte</t>
+          <t>parameter=hoogtebovenzijde, min=-8, max=325, inclusive=False</t>
         </is>
       </c>
     </row>
@@ -2884,22 +2884,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>general_003_kunstwerkopening_hoogstedoorstroombreedte</t>
+          <t>validate_001_hoogteonderzijde_plausibel</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Berekening van 'kunstwerkopening_hoogstedoorstroombreedte'</t>
+          <t>hoogteonderzijde plausibel (-8m - 325m)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
+          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>statistic=sum, related_object=kunstwerkopening, related_parameter=hoogstedoorstroombreedte</t>
+          <t>parameter=hoogteonderzijde, min=-8, max=325, inclusive=False</t>
         </is>
       </c>
     </row>
@@ -2931,17 +2931,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>validate_000_hoogtebovenzijde_plausibel</t>
+          <t>validate_002_lengte_plausibel</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>hoogtebovenzijde plausibel (-8m - 325m)</t>
+          <t>lengte plausibel (1m - 30m)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>niet-kritisch</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2956,14 +2956,14 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>parameter=hoogtebovenzijde, min=-8, max=325, inclusive=False</t>
+          <t>parameter=lengte, min=1, max=30, inclusive=False</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>brug</t>
+          <t>pomp</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2973,12 +2973,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>validate_001_hoogteonderzijde_plausibel</t>
+          <t>validate_000_capaciteit_gt_0</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>hoogteonderzijde plausibel (-8m - 325m)</t>
+          <t>De capaciteit groter dan 0</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2993,39 +2993,39 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
+          <t>GT (linkerwaarde is groter dan rechterwaarde)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>parameter=hoogteonderzijde, min=-8, max=325, inclusive=False</t>
+          <t>left=maximalecapaciteit, right=0</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>brug</t>
+          <t>gemaal</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>logische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>validate_002_lengte_plausibel</t>
+          <t>general_000_pomp_aantal_pompen</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>lengte plausibel (1m - 30m)</t>
+          <t>Berekening van 'pomp_aantal_pompen'</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>niet-kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3035,39 +3035,39 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
+          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>parameter=lengte, min=1, max=30, inclusive=False</t>
+          <t>statistic=count, related_object=pomp, fill_value=0</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>brug</t>
+          <t>gemaal</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>logische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>validate_003_laagstedoorstroombreedte_plausibel</t>
+          <t>general_001_pomp_capaciteit</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Een brug moet een plausibele laagste doorstroombreedte hebben</t>
+          <t>Berekening van 'pomp_capaciteit'</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3077,19 +3077,19 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
+          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>parameter=kunstwerkopening_laagstedoorstroombreedte, min=1, max=50, inclusive=False</t>
+          <t>statistic=sum, related_object=pomp, related_parameter=maximalecapaciteit, fill_value=0</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>brug</t>
+          <t>gemaal</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3099,12 +3099,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>validate_004_hoogstedoorstroombreedte_plausibel</t>
+          <t>validate_000_aantal_pompen_gt_0</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Een brug moet een plausibele hoogste doorstroombreedte hebben</t>
+          <t>Het aantal pompen is groter dan nul</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3119,19 +3119,19 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
+          <t>GT (linkerwaarde is groter dan rechterwaarde)</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>parameter=kunstwerkopening_hoogstedoorstroombreedte, min=1, max=50, inclusive=False</t>
+          <t>left=pomp_aantal_pompen, right=0</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>pomp</t>
+          <t>gemaal</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3141,12 +3141,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>validate_000_capaciteit_gt_0</t>
+          <t>validate_001_capaciteit_gt_0</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>De capaciteit groter dan 0</t>
+          <t>Totale capaciteit is groter dan nul</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>left=maximalecapaciteit, right=0</t>
+          <t>left=pomp_capaciteit, right=0</t>
         </is>
       </c>
     </row>
@@ -3178,22 +3178,22 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>topologische validatie</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>general_000_pomp_aantal_pompen</t>
+          <t>validate_002_geen_overlap</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Berekening van 'pomp_aantal_pompen'</t>
+          <t>Een gemaal zal geen overlap met een ander gemaal hebben</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3203,39 +3203,39 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
+          <t>not_overlapping</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>statistic=count, related_object=pomp, fill_value=0</t>
+          <t>tolerance=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>gemaal</t>
+          <t>hydroobject</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>topologische validatie</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>general_001_pomp_capaciteit</t>
+          <t>validate_000_lengte_gt_1m</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Berekening van 'pomp_capaciteit'</t>
+          <t>Hydroobject heeft voldoende lengte voor modelverwerking</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3245,34 +3245,34 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>object_relation (aggregatiewaarde ophalen uit gerelateerde objecttabel)</t>
+          <t>geometry_length</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>statistic=sum, related_object=pomp, related_parameter=maximalecapaciteit, fill_value=0</t>
+          <t>length=1, statistic=min</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>gemaal</t>
+          <t>hydroobject</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>logische validatie</t>
+          <t>topologische validatie</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>validate_000_aantal_pompen_gt_0</t>
+          <t>validate_001_goed_gesplitst</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Het aantal pompen is groter dan nul</t>
+          <t>Een hydroobject wordt gescheiden bij een samenkomst of opsplitsing</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3287,34 +3287,34 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>GT (linkerwaarde is groter dan rechterwaarde)</t>
+          <t>splitted_at_junction</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>left=pomp_aantal_pompen, right=0</t>
+          <t>tolerance=0.01</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>gemaal</t>
+          <t>hydroobject</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>logische validatie</t>
+          <t>topologische validatie</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>validate_001_capaciteit_gt_0</t>
+          <t>validate_002_goede_kruising</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Totale capaciteit is groter dan nul</t>
+          <t>Hydroobject kruist zichzelf alleen in combinatie met een duikersifonhevel of aquaduct</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3329,19 +3329,19 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>GT (linkerwaarde is groter dan rechterwaarde)</t>
+          <t>structures_at_intersections</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>left=pomp_capaciteit, right=0</t>
+          <t>tolerance=0.01, structures=duikersifonhevel</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>gemaal</t>
+          <t>hydroobject</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>validate_002_geen_overlap</t>
+          <t>validate_003_geen_eindpunt</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Een gemaal zal geen overlap met een ander gemaal hebben</t>
+          <t>Hydroobject vormt een consistent geheel, er zijn geen "doodlopende" routes</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>not_overlapping</t>
+          <t>no_dangling_node (hydroobject-eindpunt is verbonden met beginpunt van een ander hydroobject)</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>tolerance=1</t>
+          <t>tolerance=0.01</t>
         </is>
       </c>
     </row>
@@ -3393,12 +3393,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>validate_000_lengte_gt_1m</t>
+          <t>validate_004_kunstwerk_op_grens_peilgebiedpraktijk</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Hydroobject heeft voldoende lengte voor modelverwerking</t>
+          <t>Waar een hydroobject een grens van een peilgebiedpraktijk doorkruist, moet een peilscheidend kunstwerk liggen</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>geometry_length</t>
+          <t>structures_at_boundaries</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>length=1, statistic=min</t>
+          <t>areas=peilgebiedpraktijk, structures=gemaal, stuw, duikersifonhevel, tolerance=0.01, distance=25</t>
         </is>
       </c>
     </row>
@@ -3435,12 +3435,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>validate_001_goed_gesplitst</t>
+          <t>validate_005_kunstwerk_tussen_hobject</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Een hydroobject wordt gescheiden bij een samenkomst of opsplitsing</t>
+          <t>Een stuw, gemaal of bodemval moet een hydroobject opsplitsen</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>splitted_at_junction</t>
+          <t>structures_at_nodes</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>tolerance=0.01</t>
+          <t>structures=gemaal, stuw, bodemval, tolerance=1</t>
         </is>
       </c>
     </row>
@@ -3477,12 +3477,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>validate_002_goede_kruising</t>
+          <t>validate_006_kunstwerk_op_grens_peilafwijkinggebied</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Hydroobject kruist zichzelf alleen in combinatie met een duikersifonhevel of aquaduct</t>
+          <t>Waar een hydroobject een grens van een peilafwijkinggebied doorkruist, moet een peilscheidend kunstwerk liggen</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3497,39 +3497,39 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>structures_at_intersections</t>
+          <t>structures_at_boundaries</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>tolerance=0.01, structures=duikersifonhevel</t>
+          <t>areas=peilafwijkinggebied, structures=gemaal, stuw, duikersifonhevel, tolerance=0.01, distance=25</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>hydroobject</t>
+          <t>sturing</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>topologische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>validate_003_geen_eindpunt</t>
+          <t>general_000_pomp_pompcapaciteit_m3min</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Hydroobject vormt een consistent geheel, er zijn geen "doodlopende" routes</t>
+          <t>Berekening van 'pomp_pompcapaciteit_m3min'</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3539,39 +3539,39 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>no_dangling_node (hydroobject-eindpunt is verbonden met beginpunt van een ander hydroobject)</t>
+          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>tolerance=0.01</t>
+          <t>join_object=pomp, join_parameter=maximalecapaciteit, fill_value=0</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>hydroobject</t>
+          <t>sturing</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>topologische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>validate_004_kunstwerk_op_grens_peilgebiedpraktijk</t>
+          <t>general_001_pomp_pompcapaciteit_m3s</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Waar een hydroobject een grens van een peilgebiedpraktijk doorkruist, moet een peilscheidend kunstwerk liggen</t>
+          <t>Berekening van 'pomp_pompcapaciteit_m3s'</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3581,39 +3581,39 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>structures_at_boundaries</t>
+          <t>divide (quotiënt van linker- en rechterwaarde)</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>areas=peilgebiedpraktijk, structures=gemaal, stuw, duikersifonhevel, tolerance=0.01, distance=25</t>
+          <t>left=pomp_pompcapaciteit_m3min, right=60</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>hydroobject</t>
+          <t>sturing</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>topologische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>validate_005_kunstwerk_tussen_hobject</t>
+          <t>general_002_hoogteopening</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Een stuw, gemaal of bodemval moet een hydroobject opsplitsen</t>
+          <t>Berekening van 'hoogteopening'</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3623,39 +3623,39 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>structures_at_nodes</t>
+          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>structures=gemaal, stuw, bodemval, tolerance=1</t>
+          <t>join_object=regelmiddel, join_parameter=hoogteopening, fill_value=0</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>hydroobject</t>
+          <t>sturing</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>topologische validatie</t>
+          <t>algemene berekening</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>validate_006_kunstwerk_op_grens_peilafwijkinggebied</t>
+          <t>general_003_minimalehoogtebovenkant</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Waar een hydroobject een grens van een peilafwijkinggebied doorkruist, moet een peilscheidend kunstwerk liggen</t>
+          <t>Berekening van 'minimalehoogtebovenkant'</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>kritisch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>structures_at_boundaries</t>
+          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>areas=peilafwijkinggebied, structures=gemaal, stuw, duikersifonhevel, tolerance=0.01, distance=25</t>
+          <t>join_object=regelmiddel, join_parameter=minimalehoogtebovenkant, fill_value=0</t>
         </is>
       </c>
     </row>
@@ -3687,12 +3687,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>general_000_pomp_pompcapaciteit_m3min</t>
+          <t>general_004_maximalehoogtebovenkant</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Berekening van 'pomp_pompcapaciteit_m3min'</t>
+          <t>Berekening van 'maximalehoogtebovenkant'</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>join_object=pomp, join_parameter=maximalecapaciteit, fill_value=0</t>
+          <t>join_object=regelmiddel, join_parameter=maximalehoogtebovenkant, fill_value=0</t>
         </is>
       </c>
     </row>
@@ -3724,22 +3724,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>general_001_pomp_pompcapaciteit_m3s</t>
+          <t>validate_000_periode_consistent</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Berekening van 'pomp_pompcapaciteit_m3s'</t>
+          <t>Er mag geen overlap of gat in de periode zitten van meerdere sturingen met dezelfde prioriteit per gestuurd object</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3749,12 +3749,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>divide (quotiënt van linker- en rechterwaarde)</t>
+          <t>consistent_period</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>left=pomp_pompcapaciteit_m3min, right=60</t>
+          <t>max_gap=1</t>
         </is>
       </c>
     </row>
@@ -3766,37 +3766,37 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>general_002_hoogteopening</t>
+          <t>validate_001_pomp_bestaat</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Berekening van 'hoogteopening'</t>
+          <t>de gestuurde pomp moet bestaan</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>pompid NOTNA</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
+          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>join_object=regelmiddel, join_parameter=hoogteopening, fill_value=0</t>
+          <t>join_object=pomp</t>
         </is>
       </c>
     </row>
@@ -3808,37 +3808,37 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>general_003_minimalehoogtebovenkant</t>
+          <t>validate_002_regelmiddel_bestaat</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Berekening van 'minimalehoogtebovenkant'</t>
+          <t>het regelmiddel moet bestaan</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>regelmiddelid NOTNA</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
+          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>join_object=regelmiddel, join_parameter=minimalehoogtebovenkant, fill_value=0</t>
+          <t>join_object=regelmiddel</t>
         </is>
       </c>
     </row>
@@ -3850,37 +3850,37 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>algemene berekening</t>
+          <t>logische validatie</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>general_004_maximalehoogtebovenkant</t>
+          <t>validate_003_hydrologische_rvw_bestaat</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Berekening van 'maximalehoogtebovenkant'</t>
+          <t>de gestuurde hydrologische randvoorwaarde moet bestaan</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kritisch</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>hydrologischerandvoorwaardeid NOTNA</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>join_parameter (koppeling met parameter uit ander objecttabel)</t>
+          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>join_object=regelmiddel, join_parameter=maximalehoogtebovenkant, fill_value=0</t>
+          <t>join_object=hydrologischerandvoorwaarde</t>
         </is>
       </c>
     </row>
@@ -3897,12 +3897,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>validate_000_periode_consistent</t>
+          <t>validate_004_vastewaarde_pmp_binnen_bereik</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Er mag geen overlap of gat in de periode zitten van meerdere sturingen met dezelfde prioriteit per gestuurd object</t>
+          <t>vaste waarde pomp zal binnen het fysieke bereik van de stuurvariabele passen</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3912,17 +3912,17 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>stuurvariabele ISIN (pompdebiet)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>consistent_period</t>
+          <t>LE (linkerwaarde is minder dan of gelijk aan rechterwaarde)</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>max_gap=1</t>
+          <t>left=vastewaarde, right=pomp_pompcapaciteit_m3s</t>
         </is>
       </c>
     </row>
@@ -3939,12 +3939,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>validate_001_pomp_bestaat</t>
+          <t>validate_005_vastewaarde_onderlaat_binnen_bereik</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>de gestuurde pomp moet bestaan</t>
+          <t>vaste waarde onderlaat zal binnen het fysieke bereik van de stuurvariabele passen</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3954,17 +3954,17 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>pompid NOTNA</t>
+          <t>stuurvariabele ISIN (hoogte opening)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
+          <t>LE (linkerwaarde is minder dan of gelijk aan rechterwaarde)</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>join_object=pomp</t>
+          <t>left=vastewaarde, right=hoogteopening</t>
         </is>
       </c>
     </row>
@@ -3981,12 +3981,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>validate_002_regelmiddel_bestaat</t>
+          <t>validate_006_vastewaarde_overlaat_binnen_bereik</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>het regelmiddel moet bestaan</t>
+          <t>vaste waarde overlaat zal binnen het fysieke bereik van de stuurvariabele passen</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3996,17 +3996,17 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>regelmiddelid NOTNA</t>
+          <t>stuurvariabele ISIN (bovenkant afsluitmiddel,)</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
+          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>join_object=regelmiddel</t>
+          <t>parameter=vastewaarde, min=minimalehoogtebovenkant, max=maximalehoogtebovenkant, inclusive=True</t>
         </is>
       </c>
     </row>
@@ -4023,12 +4023,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>validate_003_hydrologische_rvw_bestaat</t>
+          <t>validate_007_pmp_juiste_stuurvariabele</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>de gestuurde hydrologische randvoorwaarde moet bestaan</t>
+          <t>gestuurde pomp heeft juiste stuurvariabele</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4038,17 +4038,17 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>hydrologischerandvoorwaardeid NOTNA</t>
+          <t>pompid NOTNA</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>join_object_exists (object komt voor in de gerelateerde objecttabel)</t>
+          <t>ISIN (waarde komt voor in lijst)</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>join_object=hydrologischerandvoorwaarde</t>
+          <t>parameter=stuurvariabele, array=pompdebiet</t>
         </is>
       </c>
     </row>
@@ -4065,12 +4065,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>validate_004_vastewaarde_pmp_binnen_bereik</t>
+          <t>validate_008_regelmiddel_juiste_stuurvariabele</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>vaste waarde pomp zal binnen het fysieke bereik van de stuurvariabele passen</t>
+          <t>gestuurde regelmiddel heeft juiste stuurvariabele</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4080,190 +4080,22 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>stuurvariabele ISIN (pompdebiet)</t>
+          <t>regelmiddelid NOTNA</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>LE (linkerwaarde is minder dan of gelijk aan rechterwaarde)</t>
+          <t>ISIN (waarde komt voor in lijst)</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>left=vastewaarde, right=pomp_pompcapaciteit_m3s</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>sturing</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>logische validatie</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>validate_005_vastewaarde_onderlaat_binnen_bereik</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>vaste waarde onderlaat zal binnen het fysieke bereik van de stuurvariabele passen</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>kritisch</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>stuurvariabele ISIN (hoogte opening)</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>LE (linkerwaarde is minder dan of gelijk aan rechterwaarde)</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>left=vastewaarde, right=hoogteopening</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>sturing</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>logische validatie</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>validate_006_vastewaarde_overlaat_binnen_bereik</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>vaste waarde overlaat zal binnen het fysieke bereik van de stuurvariabele passen</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>kritisch</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>stuurvariabele ISIN (bovenkant afsluitmiddel,)</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>BE (waarde ligt tussen de min- en max-waarde)</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>parameter=vastewaarde, min=minimalehoogtebovenkant, max=maximalehoogtebovenkant, inclusive=True</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>sturing</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>logische validatie</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>validate_007_pmp_juiste_stuurvariabele</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>gestuurde pomp heeft juiste stuurvariabele</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>kritisch</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>pompid NOTNA</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>ISIN (waarde komt voor in lijst)</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>parameter=stuurvariabele, array=pompdebiet</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>sturing</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>logische validatie</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>validate_008_regelmiddel_juiste_stuurvariabele</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>gestuurde regelmiddel heeft juiste stuurvariabele</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>kritisch</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>regelmiddelid NOTNA</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>ISIN (waarde komt voor in lijst)</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
           <t>parameter=stuurvariabele, array=bovenkant afsluitmiddel,, hoogte opening</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H91"/>
+  <autoFilter ref="A1:H87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>